<commit_message>
update: thay doi nguon danh sach san pham sang lay tu tbl_baophu_nv_92
</commit_message>
<xml_diff>
--- a/public/templates/template_bao_cao_phan_tich_diem_ban_do_phu.xlsx
+++ b/public/templates/template_bao_cao_phan_tich_diem_ban_do_phu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Local Google Drive\web_v4_skill\web_v4_pro\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F33C4721-37ED-455A-8D5D-0642764CD45D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162E4506-734A-4141-90B0-DFC10D0133AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15943" xr2:uid="{863BF2B5-95BA-4E61-A056-7F3F8812E416}"/>
   </bookViews>
@@ -235,7 +235,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -271,6 +271,9 @@
     </xf>
     <xf numFmtId="41" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -612,7 +615,7 @@
   <cols>
     <col min="1" max="1" width="7.28515625" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="28.92578125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="28.92578125" style="14" customWidth="1"/>
     <col min="4" max="4" width="12.640625" style="5" customWidth="1"/>
     <col min="5" max="5" width="26.0703125" style="9" customWidth="1"/>
     <col min="6" max="6" width="5.5" style="5" bestFit="1" customWidth="1"/>
@@ -668,6 +671,9 @@
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
     </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C5" s="9"/>
+    </row>
     <row r="6" spans="1:8" s="8" customFormat="1" ht="37.299999999999997" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>3</v>

</xml_diff>